<commit_message>
Corrected symbol reference for Luminous Efficacy
</commit_message>
<xml_diff>
--- a/CUQ/_docs/SI_Constants.xlsx
+++ b/CUQ/_docs/SI_Constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10709"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/Semantic-SI/CUQ/_docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh25\git\SI-Reference-Point-2023\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE890F9C-8107-CB40-9363-47CD6F5262E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454BEBE2-C92F-4639-B61C-7D9BBEAA0D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2080" yWindow="3080" windowWidth="25260" windowHeight="16760" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -179,7 +179,7 @@
     <t>symbol codes defined in 'notes.xlsx'</t>
   </si>
   <si>
-    <t>@lpws@</t>
+    <t>@lecs@</t>
   </si>
 </sst>
 </file>
@@ -533,15 +533,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9DD0E9-1DD4-4C4F-AE4A-1F84A9440AB2}">
   <dimension ref="A1:H8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="34.5" customWidth="1"/>
     <col min="3" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="6" width="17.6640625" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="1"/>
+    <col min="5" max="6" width="17.640625" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -567,7 +567,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -593,7 +593,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -616,7 +616,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -639,7 +639,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -662,7 +662,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -685,7 +685,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -708,7 +708,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
SI-Reference-Point-2023-9 Updates to constants TTL file needed
Added/updated the following:
- added predicates hasDatatype, hasValueAsString, and hasUpdatedDate to CUQ_TBox.py
- added data for datatypes, values as strings, and updated date to the SI_Constants.xlsx file
- added code to Constants_ABox.py to add the additional data above
- minor code formatting updates
- updated dates all set to "2018-05-20" - some will require update
</commit_message>
<xml_diff>
--- a/CUQ/_docs/SI_Constants.xlsx
+++ b/CUQ/_docs/SI_Constants.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jh25\git\SI-Reference-Point-2023\CUQ\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{454BEBE2-C92F-4639-B61C-7D9BBEAA0D28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A927843-DBDF-6B4D-8BA4-E11034A6FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
+    <workbookView xWindow="14040" yWindow="500" windowWidth="29040" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="61">
   <si>
     <t>Avogadro constant</t>
   </si>
@@ -110,9 +110,6 @@
     <t>efficacité lumineuse</t>
   </si>
   <si>
-    <t>Symbole</t>
-  </si>
-  <si>
     <t>unit</t>
   </si>
   <si>
@@ -173,19 +170,66 @@
     <t>@avos@</t>
   </si>
   <si>
-    <t>Comments</t>
-  </si>
-  <si>
     <t>symbol codes defined in 'notes.xlsx'</t>
   </si>
   <si>
     <t>@lecs@</t>
+  </si>
+  <si>
+    <t>value_str</t>
+  </si>
+  <si>
+    <t>9 192 631 770</t>
+  </si>
+  <si>
+    <t>299 792 458</t>
+  </si>
+  <si>
+    <t>683</t>
+  </si>
+  <si>
+    <t>value_type</t>
+  </si>
+  <si>
+    <t>xsd:integer</t>
+  </si>
+  <si>
+    <t>xsd:double</t>
+  </si>
+  <si>
+    <t>symbol</t>
+  </si>
+  <si>
+    <t>comments</t>
+  </si>
+  <si>
+    <t>updateddate</t>
+  </si>
+  <si>
+    <t>2018-05-20</t>
+  </si>
+  <si>
+    <t>1.380 649 x 10⁻²³</t>
+  </si>
+  <si>
+    <t>1.602 176 634 x 10⁻¹⁹</t>
+  </si>
+  <si>
+    <t>6.626 070 15 x 10³⁴</t>
+  </si>
+  <si>
+    <t>6.022 140 76 x 10²³</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.000000E+00"/>
+    <numFmt numFmtId="166" formatCode="0.00000000E+00"/>
+    <numFmt numFmtId="167" formatCode="0.000000000E+00"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -215,9 +259,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,21 +579,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9DD0E9-1DD4-4C4F-AE4A-1F84A9440AB2}">
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15.9" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="34.5" customWidth="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="6" width="17.640625" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" style="1"/>
+    <col min="10" max="10" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
         <v>5</v>
@@ -555,24 +607,33 @@
         <v>6</v>
       </c>
       <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" t="s">
-        <v>45</v>
+      <c r="I1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
@@ -580,20 +641,29 @@
       <c r="D2" t="s">
         <v>20</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2">
         <v>9192631770</v>
       </c>
-      <c r="F2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="H2" t="s">
-        <v>46</v>
+        <v>25</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="K2" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -601,27 +671,36 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3">
         <v>299792458</v>
       </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>40</v>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -629,17 +708,26 @@
       <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" s="3">
         <v>6.6260701499999998E-34</v>
       </c>
-      <c r="F4" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>41</v>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -652,22 +740,31 @@
       <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" s="4">
         <v>1.6021766339999999E-19</v>
       </c>
-      <c r="F5" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>42</v>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
         <v>1</v>
@@ -675,22 +772,31 @@
       <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="2">
         <v>1.3806490000000001E-23</v>
       </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>43</v>
+      <c r="H6" t="s">
+        <v>29</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
         <v>0</v>
@@ -698,17 +804,26 @@
       <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" s="3">
         <v>6.0221407599999999E+23</v>
       </c>
-      <c r="F7" t="s">
-        <v>31</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>44</v>
+      <c r="H7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -721,17 +836,29 @@
       <c r="D8" t="s">
         <v>23</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8">
         <v>683</v>
       </c>
-      <c r="F8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>47</v>
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="F8" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
SI-Reference-Point-2023-13 on the revised constants file
Addition of string version of units for the defining constants
</commit_message>
<xml_diff>
--- a/CUQ/_docs/SI_Constants.xlsx
+++ b/CUQ/_docs/SI_Constants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A927843-DBDF-6B4D-8BA4-E11034A6FBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AD171C-5A9A-6C4E-AEC4-98DF465B3219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14040" yWindow="500" windowWidth="29040" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="67">
   <si>
     <t>Avogadro constant</t>
   </si>
@@ -219,6 +219,24 @@
   </si>
   <si>
     <t>6.022 140 76 x 10²³</t>
+  </si>
+  <si>
+    <t>unit_str</t>
+  </si>
+  <si>
+    <t>m s⁻¹</t>
+  </si>
+  <si>
+    <t>J s</t>
+  </si>
+  <si>
+    <t>J K⁻¹</t>
+  </si>
+  <si>
+    <t>mol⁻¹</t>
+  </si>
+  <si>
+    <t>lm W⁻¹</t>
   </si>
 </sst>
 </file>
@@ -227,8 +245,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000E+00"/>
-    <numFmt numFmtId="166" formatCode="0.00000000E+00"/>
-    <numFmt numFmtId="167" formatCode="0.000000000E+00"/>
+    <numFmt numFmtId="165" formatCode="0.00000000E+00"/>
+    <numFmt numFmtId="166" formatCode="0.000000000E+00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -263,8 +281,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9DD0E9-1DD4-4C4F-AE4A-1F84A9440AB2}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
@@ -588,12 +606,12 @@
     <col min="5" max="5" width="12.6640625" customWidth="1"/>
     <col min="6" max="6" width="19.1640625" customWidth="1"/>
     <col min="7" max="7" width="17.6640625" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" style="1"/>
-    <col min="10" max="10" width="13" style="1" customWidth="1"/>
+    <col min="8" max="9" width="10.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="1"/>
+    <col min="11" max="11" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -618,17 +636,20 @@
       <c r="H1" t="s">
         <v>24</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -654,16 +675,19 @@
         <v>25</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -689,13 +713,16 @@
         <v>27</v>
       </c>
       <c r="I3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -721,13 +748,16 @@
         <v>28</v>
       </c>
       <c r="I4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -753,13 +783,16 @@
         <v>26</v>
       </c>
       <c r="I5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -785,13 +818,16 @@
         <v>29</v>
       </c>
       <c r="I6" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -817,13 +853,16 @@
         <v>30</v>
       </c>
       <c r="I7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -849,9 +888,12 @@
         <v>31</v>
       </c>
       <c r="I8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix constant update dates and include defining resolution column
</commit_message>
<xml_diff>
--- a/CUQ/_docs/SI_Constants.xlsx
+++ b/CUQ/_docs/SI_Constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07AD171C-5A9A-6C4E-AEC4-98DF465B3219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F96CDB-E8B8-4561-A733-2081FAAA69DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14040" yWindow="500" windowWidth="29040" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>Avogadro constant</t>
   </si>
@@ -206,9 +206,6 @@
     <t>updateddate</t>
   </si>
   <si>
-    <t>2018-05-20</t>
-  </si>
-  <si>
     <t>1.380 649 x 10⁻²³</t>
   </si>
   <si>
@@ -237,6 +234,33 @@
   </si>
   <si>
     <t>lm W⁻¹</t>
+  </si>
+  <si>
+    <t>1975-06-03</t>
+  </si>
+  <si>
+    <t>1967-10-13</t>
+  </si>
+  <si>
+    <t>1979-10-11</t>
+  </si>
+  <si>
+    <t>2019-05-20</t>
+  </si>
+  <si>
+    <t>hasDefiningResolution</t>
+  </si>
+  <si>
+    <t>CGPM13-Res1</t>
+  </si>
+  <si>
+    <t>CGPM16-Res3</t>
+  </si>
+  <si>
+    <t>CGPM26-Res1</t>
+  </si>
+  <si>
+    <t>CGPM15-Res2</t>
   </si>
 </sst>
 </file>
@@ -285,7 +309,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -301,7 +325,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -597,21 +621,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9DD0E9-1DD4-4C4F-AE4A-1F84A9440AB2}">
-  <dimension ref="A1:L8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:M8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="1" max="1" width="20.375" customWidth="1"/>
+    <col min="2" max="2" width="18.875" customWidth="1"/>
     <col min="3" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="19.1640625" customWidth="1"/>
-    <col min="7" max="7" width="17.6640625" customWidth="1"/>
-    <col min="8" max="9" width="10.33203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="1"/>
+    <col min="5" max="5" width="12.625" customWidth="1"/>
+    <col min="6" max="6" width="19.125" customWidth="1"/>
+    <col min="7" max="7" width="17.625" customWidth="1"/>
+    <col min="8" max="9" width="10.375" customWidth="1"/>
+    <col min="10" max="10" width="10.875" style="1"/>
     <col min="11" max="11" width="13" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -637,7 +663,7 @@
         <v>24</v>
       </c>
       <c r="I1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>53</v>
@@ -645,11 +671,14 @@
       <c r="K1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="M1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -681,13 +710,16 @@
         <v>38</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -713,16 +745,19 @@
         <v>27</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>39</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>56</v>
+        <v>66</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -739,7 +774,7 @@
         <v>52</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G4" s="3">
         <v>6.6260701499999998E-34</v>
@@ -748,16 +783,19 @@
         <v>28</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>40</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -774,7 +812,7 @@
         <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5" s="4">
         <v>1.6021766339999999E-19</v>
@@ -789,10 +827,13 @@
         <v>41</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -809,7 +850,7 @@
         <v>52</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6" s="2">
         <v>1.3806490000000001E-23</v>
@@ -818,16 +859,19 @@
         <v>29</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>42</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -844,7 +888,7 @@
         <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G7" s="3">
         <v>6.0221407599999999E+23</v>
@@ -853,16 +897,19 @@
         <v>30</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>43</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -888,13 +935,16 @@
         <v>31</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>45</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>56</v>
+        <v>68</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Python formatting update for Constants_ABox.py
</commit_message>
<xml_diff>
--- a/CUQ/_docs/SI_Constants.xlsx
+++ b/CUQ/_docs/SI_Constants.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gruber04\git_repos\BIPM\Semantic-SI\CUQ\_docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n00002621/PycharmProjects/SI-Reference-Point-2023/CUQ/_docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3FD3DFA-1AEB-40DC-9279-37F1B2228248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5A666D-F223-5242-87FD-09FCEC1507E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-8310" windowWidth="38640" windowHeight="21390" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
+    <workbookView xWindow="14040" yWindow="500" windowWidth="31020" windowHeight="15840" xr2:uid="{A8E124C3-E099-C041-B0C2-7CC2CA979201}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>Avogadro constant</t>
   </si>
@@ -170,9 +170,6 @@
     <t>@avos@</t>
   </si>
   <si>
-    <t>symbol codes defined in 'notes.xlsx'</t>
-  </si>
-  <si>
     <t>@lecs@</t>
   </si>
   <si>
@@ -206,6 +203,18 @@
     <t>updateddate</t>
   </si>
   <si>
+    <t>1.380 649 x 10⁻²³</t>
+  </si>
+  <si>
+    <t>1.602 176 634 x 10⁻¹⁹</t>
+  </si>
+  <si>
+    <t>6.626 070 15 x 10³⁴</t>
+  </si>
+  <si>
+    <t>6.022 140 76 x 10²³</t>
+  </si>
+  <si>
     <t>unit_str</t>
   </si>
   <si>
@@ -224,43 +233,25 @@
     <t>lm W⁻¹</t>
   </si>
   <si>
-    <t>1975-06-03</t>
-  </si>
-  <si>
-    <t>1967-10-13</t>
-  </si>
-  <si>
-    <t>1979-10-11</t>
+    <t>1975-01-01</t>
+  </si>
+  <si>
+    <t>1979-01-01</t>
   </si>
   <si>
     <t>2019-05-20</t>
   </si>
   <si>
-    <t>hasDefiningResolution</t>
-  </si>
-  <si>
-    <t>CGPM13-Res1</t>
-  </si>
-  <si>
-    <t>CGPM16-Res3</t>
-  </si>
-  <si>
-    <t>CGPM26-Res1</t>
-  </si>
-  <si>
-    <t>CGPM15-Res2</t>
-  </si>
-  <si>
-    <t>6.626 070 15 x 10⁻³⁴</t>
-  </si>
-  <si>
-    <t>1.602 176 634 x 10⁻¹⁹</t>
-  </si>
-  <si>
-    <t>1.380 649 x 10⁻²³</t>
-  </si>
-  <si>
-    <t>6.022 140 76 x 10²³</t>
+    <t>https://doi.org/10.59161/cgpm2018res1e</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.59161/cgpm1967res1e</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.59161/cgpm1979res3e</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.59161/cgpm1975res2e</t>
   </si>
 </sst>
 </file>
@@ -272,16 +263,10 @@
     <numFmt numFmtId="165" formatCode="0.00000000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000000000E+00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -307,16 +292,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -332,7 +316,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -628,331 +612,322 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F9DD0E9-1DD4-4C4F-AE4A-1F84A9440AB2}">
-  <dimension ref="A1:M8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="20.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="17.625" style="1" customWidth="1"/>
-    <col min="8" max="9" width="10.375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.875" style="2"/>
-    <col min="11" max="11" width="13" style="2" customWidth="1"/>
-    <col min="12" max="12" width="23" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="30.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="10.875" style="1"/>
+    <col min="1" max="1" width="20.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="4" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" customWidth="1"/>
+    <col min="7" max="7" width="17.6640625" customWidth="1"/>
+    <col min="8" max="9" width="10.33203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" style="1"/>
+    <col min="11" max="11" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
         <v>50</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="G2">
+        <v>9192631770</v>
+      </c>
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>54</v>
+      <c r="L2" t="s">
+        <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="1" t="s">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3">
+        <v>299792458</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" s="1">
-        <v>9192631770</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="1">
-        <v>299792458</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="G4" s="3">
         <v>6.6260701499999998E-34</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="I4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>69</v>
+      <c r="K4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>72</v>
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>56</v>
       </c>
       <c r="G5" s="4">
         <v>1.6021766339999999E-19</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>69</v>
+      <c r="K5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="5">
+      <c r="E6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="2">
         <v>1.3806490000000001E-23</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="J6" s="2" t="s">
+      <c r="I6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>69</v>
+      <c r="K6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>0</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>74</v>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>58</v>
       </c>
       <c r="G7" s="3">
         <v>6.0221407599999999E+23</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" t="s">
         <v>30</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="I7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>69</v>
+      <c r="K7" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>23</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="1">
+      <c r="E8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8">
         <v>683</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" t="s">
         <v>31</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="K8" s="2" t="s">
+      <c r="I8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>68</v>
+      <c r="J8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>